<commit_message>
various freqscan test codes
</commit_message>
<xml_diff>
--- a/Examples/AcPowerSystem/IEEE_14Bus/IEEE_14Bus.xlsx
+++ b/Examples/AcPowerSystem/IEEE_14Bus/IEEE_14Bus.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Power-System-Analysis-Toolbox\Examples\AcPowerSystem\IEEE_14Bus\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gzhan\Documents\Imperial College London\PhD Year 1\Hybrid ACDC\Simplus-Grid-Tool-2025May_HybridACDC\Simplus-Grid-Tool\Examples\AcPowerSystem\IEEE_14Bus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C711BCA9-472B-46EA-9163-D8F4DB11A35F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9237A491-D69B-4DBD-A090-BC5B9DB701B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bus" sheetId="1" r:id="rId1"/>
@@ -244,20 +244,20 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="176" formatCode="0.00_ "/>
-    <numFmt numFmtId="177" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.00_ "/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -266,7 +266,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -274,7 +274,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -282,7 +282,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -290,13 +290,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -324,13 +324,13 @@
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -612,19 +612,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L16"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="4" max="4" width="11.1328125" customWidth="1"/>
-    <col min="9" max="9" width="10.86328125" customWidth="1"/>
-    <col min="10" max="10" width="11.1328125" customWidth="1"/>
+    <col min="4" max="4" width="11.140625" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="10" max="10" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12">
       <c r="A1" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:12">
       <c r="A2" s="3" t="s">
         <v>32</v>
       </c>
@@ -662,7 +662,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:12">
       <c r="A3" s="6">
         <v>1</v>
       </c>
@@ -700,7 +700,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:12">
       <c r="A4" s="6">
         <v>2</v>
       </c>
@@ -744,7 +744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:12">
       <c r="A5" s="6">
         <v>3</v>
       </c>
@@ -786,7 +786,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:12">
       <c r="A6" s="7">
         <v>4</v>
       </c>
@@ -826,7 +826,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:12">
       <c r="A7" s="7">
         <v>5</v>
       </c>
@@ -866,7 +866,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:12">
       <c r="A8" s="6">
         <v>6</v>
       </c>
@@ -909,7 +909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:12">
       <c r="A9" s="7">
         <v>7</v>
       </c>
@@ -947,7 +947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:12">
       <c r="A10" s="6">
         <v>8</v>
       </c>
@@ -988,7 +988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:12">
       <c r="A11" s="7">
         <v>9</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:12">
       <c r="A12">
         <v>10</v>
       </c>
@@ -1068,7 +1068,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:12">
       <c r="A13">
         <v>11</v>
       </c>
@@ -1108,7 +1108,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:12">
       <c r="A14">
         <v>12</v>
       </c>
@@ -1148,7 +1148,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:12">
       <c r="A15">
         <v>13</v>
       </c>
@@ -1188,7 +1188,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:12">
       <c r="A16">
         <v>14</v>
       </c>
@@ -1238,30 +1238,30 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34645F5B-1D7A-4323-9AD6-5FF81941CA24}">
   <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.86328125" customWidth="1"/>
-    <col min="2" max="2" width="29.59765625" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" customWidth="1"/>
+    <col min="2" max="2" width="29.5703125" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="15.1328125" customWidth="1"/>
-    <col min="5" max="5" width="12.3984375" customWidth="1"/>
-    <col min="6" max="6" width="13.59765625" customWidth="1"/>
-    <col min="7" max="7" width="13.86328125" customWidth="1"/>
-    <col min="8" max="8" width="15.1328125" customWidth="1"/>
-    <col min="9" max="9" width="18.86328125" customWidth="1"/>
-    <col min="10" max="10" width="18.59765625" customWidth="1"/>
-    <col min="11" max="11" width="17.1328125" customWidth="1"/>
-    <col min="12" max="12" width="17.86328125" customWidth="1"/>
-    <col min="13" max="13" width="14.3984375" customWidth="1"/>
-    <col min="14" max="14" width="13.1328125" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" customWidth="1"/>
+    <col min="8" max="8" width="15.140625" customWidth="1"/>
+    <col min="9" max="9" width="18.85546875" customWidth="1"/>
+    <col min="10" max="10" width="18.5703125" customWidth="1"/>
+    <col min="11" max="11" width="17.140625" customWidth="1"/>
+    <col min="12" max="12" width="17.85546875" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" customWidth="1"/>
+    <col min="14" max="14" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10">
       <c r="A1" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10">
       <c r="A2" s="3" t="s">
         <v>19</v>
       </c>
@@ -1272,7 +1272,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10">
       <c r="A3" s="7">
         <v>1</v>
       </c>
@@ -1296,7 +1296,7 @@
       <c r="I3" s="8"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:10">
       <c r="A4" s="7">
         <v>2</v>
       </c>
@@ -1320,7 +1320,7 @@
       <c r="I4" s="8"/>
       <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:10">
       <c r="A5" s="7">
         <v>3</v>
       </c>
@@ -1343,7 +1343,7 @@
       <c r="H5" s="8"/>
       <c r="I5" s="8"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:10">
       <c r="A6" s="7">
         <v>6</v>
       </c>
@@ -1366,7 +1366,7 @@
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:10">
       <c r="A7" s="7">
         <v>8</v>
       </c>
@@ -1399,33 +1399,33 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64D00B5E-E2E7-41B8-8388-8931D474EA96}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="5" max="5" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.59765625" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7">
       <c r="A1" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7">
       <c r="A3" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7">
       <c r="A4" s="3" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7">
       <c r="A5" s="3" t="s">
         <v>35</v>
       </c>
@@ -1448,7 +1448,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7">
       <c r="A6">
         <v>1</v>
       </c>
@@ -1472,7 +1472,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1496,7 +1496,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7">
       <c r="A8">
         <v>2</v>
       </c>
@@ -1520,7 +1520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7">
       <c r="A9">
         <v>2</v>
       </c>
@@ -1544,7 +1544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7">
       <c r="A10">
         <v>2</v>
       </c>
@@ -1568,7 +1568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7">
       <c r="A11">
         <v>3</v>
       </c>
@@ -1592,7 +1592,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7">
       <c r="A12">
         <v>4</v>
       </c>
@@ -1615,7 +1615,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7">
       <c r="A13">
         <v>4</v>
       </c>
@@ -1638,7 +1638,7 @@
         <v>0.97799999999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7">
       <c r="A14">
         <v>4</v>
       </c>
@@ -1661,7 +1661,7 @@
         <v>0.96899999999999997</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7">
       <c r="A15">
         <v>5</v>
       </c>
@@ -1684,7 +1684,7 @@
         <v>0.93200000000000005</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7">
       <c r="A16">
         <v>6</v>
       </c>
@@ -1707,7 +1707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:7">
       <c r="A17">
         <v>6</v>
       </c>
@@ -1730,7 +1730,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:7">
       <c r="A18">
         <v>6</v>
       </c>
@@ -1753,7 +1753,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:7">
       <c r="A19">
         <v>7</v>
       </c>
@@ -1776,7 +1776,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:7">
       <c r="A20">
         <v>7</v>
       </c>
@@ -1799,7 +1799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:7">
       <c r="A21">
         <v>9</v>
       </c>
@@ -1822,7 +1822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:7">
       <c r="A22">
         <v>9</v>
       </c>
@@ -1845,7 +1845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:7">
       <c r="A23">
         <v>10</v>
       </c>
@@ -1868,7 +1868,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:7">
       <c r="A24">
         <v>12</v>
       </c>
@@ -1891,7 +1891,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:7">
       <c r="A25">
         <v>13</v>
       </c>
@@ -1914,7 +1914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:7">
       <c r="A26">
         <v>9</v>
       </c>
@@ -1947,18 +1947,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B0C2B6E-74BD-40FA-8EB6-D64D8C21837A}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="7" max="7" width="14.86328125" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7">
       <c r="A2" s="3" t="s">
         <v>35</v>
       </c>
@@ -1991,29 +1991,28 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EB93A31-1E5A-4104-8C10-8E6599437516}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="18.59765625" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="15.86328125" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2">
       <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2">
       <c r="A2" s="5" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="1">
-        <f>B3*500</f>
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>29</v>
       </c>
@@ -2021,7 +2020,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -2029,7 +2028,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -2047,17 +2046,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EFCB373-2341-40B6-A375-7BA50357479A}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30.1328125" customWidth="1"/>
+    <col min="1" max="1" width="30.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" s="3" t="s">
         <v>38</v>
       </c>
@@ -2066,7 +2065,7 @@
       </c>
       <c r="C2" s="3"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -2074,7 +2073,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -2082,7 +2081,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -2090,7 +2089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -2098,7 +2097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -2106,7 +2105,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -2114,7 +2113,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -2122,7 +2121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -2130,7 +2129,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -2138,7 +2137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>41</v>
       </c>

</xml_diff>